<commit_message>
Data. Italy and Germany
</commit_message>
<xml_diff>
--- a/main_find_best_hyper/data/italy/2024-07-25/df_iteration.xlsx
+++ b/main_find_best_hyper/data/italy/2024-07-25/df_iteration.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AL40"/>
+  <dimension ref="A1:AL52"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -5648,6 +5648,1578 @@
       <c r="AK40" t="inlineStr"/>
       <c r="AL40" t="inlineStr"/>
     </row>
+    <row r="41">
+      <c r="A41" t="n">
+        <v>62</v>
+      </c>
+      <c r="B41" t="n">
+        <v>30</v>
+      </c>
+      <c r="C41" t="n">
+        <v>3</v>
+      </c>
+      <c r="D41" t="b">
+        <v>1</v>
+      </c>
+      <c r="E41" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="F41" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="G41" t="n">
+        <v>10</v>
+      </c>
+      <c r="H41" t="inlineStr">
+        <is>
+          <t>[771, 772, 773]</t>
+        </is>
+      </c>
+      <c r="I41" t="inlineStr"/>
+      <c r="J41" t="inlineStr">
+        <is>
+          <t>under</t>
+        </is>
+      </c>
+      <c r="K41" t="n">
+        <v>0.125</v>
+      </c>
+      <c r="L41" t="n">
+        <v>0.125</v>
+      </c>
+      <c r="M41" t="inlineStr">
+        <is>
+          <t>(1161, 16)</t>
+        </is>
+      </c>
+      <c r="N41" t="inlineStr">
+        <is>
+          <t>(258, 16)</t>
+        </is>
+      </c>
+      <c r="O41" t="inlineStr">
+        <is>
+          <t>(258, 16)</t>
+        </is>
+      </c>
+      <c r="P41" t="inlineStr">
+        <is>
+          <t>['id_team_away', 'is_cup', 'h2h_35', 'h2h_3_segun_loc', 'h2h_3', 'dif_mean_last_match_goals', 'dif_mean_last_match_goals_against', 'dif_mean_last_match_ball_possession', 'dif_mean_last_match_shots_on_goal', 'dif_mean_last_match_goal_attempts', 'dif_mean_last_match_goal_attempts_against', 'dif_n_player_miss', 'dif_mean_age_player_start', 'dif_mean_hei_player_sub', 'dif_mean_hei_player_miss', 'dif_mean_rat_player_start']</t>
+        </is>
+      </c>
+      <c r="Q41" t="n">
+        <v>10</v>
+      </c>
+      <c r="R41" t="n">
+        <v>54.65116279069767</v>
+      </c>
+      <c r="S41" t="n">
+        <v>50.34865829304756</v>
+      </c>
+      <c r="T41" t="n">
+        <v>50.94202721321365</v>
+      </c>
+      <c r="U41" t="n">
+        <v>62.4031007751938</v>
+      </c>
+      <c r="V41" t="n">
+        <v>-7.751937984496131</v>
+      </c>
+      <c r="W41" t="n">
+        <v>0.02103678954097774</v>
+      </c>
+      <c r="X41" t="n">
+        <v>-0.01561418257570409</v>
+      </c>
+      <c r="Y41" t="n">
+        <v>-0.02816219586786872</v>
+      </c>
+      <c r="Z41" t="n">
+        <v>0.05940368256978296</v>
+      </c>
+      <c r="AA41" t="n">
+        <v>0.8146255580860639</v>
+      </c>
+      <c r="AB41" t="n">
+        <v>0.003157463403434356</v>
+      </c>
+      <c r="AC41" t="n">
+        <v>-0.15</v>
+      </c>
+      <c r="AD41" t="inlineStr">
+        <is>
+          <t>equal</t>
+        </is>
+      </c>
+      <c r="AE41" t="inlineStr">
+        <is>
+          <t>(0, 0)</t>
+        </is>
+      </c>
+      <c r="AF41" t="inlineStr">
+        <is>
+          <t>(1, 0)</t>
+        </is>
+      </c>
+      <c r="AG41" t="inlineStr">
+        <is>
+          <t>LogisticRegression</t>
+        </is>
+      </c>
+      <c r="AH41" t="inlineStr">
+        <is>
+          <t>{'C': 0.1, 'class_weight': None, 'dual': False, 'fit_intercept': True, 'intercept_scaling': 1, 'l1_ratio': None, 'max_iter': 1000, 'multi_class': 'auto', 'n_jobs': None, 'penalty': 'l1', 'random_state': None, 'solver': 'liblinear', 'tol': 0.0001, 'verbose': 0, 'warm_start': False}</t>
+        </is>
+      </c>
+      <c r="AI41" t="n">
+        <v>31.37931034482759</v>
+      </c>
+      <c r="AJ41" t="n">
+        <v>0.003967683611701261</v>
+      </c>
+      <c r="AK41" t="inlineStr"/>
+      <c r="AL41" t="inlineStr"/>
+    </row>
+    <row r="42">
+      <c r="A42" t="n">
+        <v>63</v>
+      </c>
+      <c r="B42" t="n">
+        <v>30</v>
+      </c>
+      <c r="C42" t="n">
+        <v>3</v>
+      </c>
+      <c r="D42" t="b">
+        <v>1</v>
+      </c>
+      <c r="E42" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="F42" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="G42" t="n">
+        <v>10</v>
+      </c>
+      <c r="H42" t="inlineStr">
+        <is>
+          <t>[771, 772, 773]</t>
+        </is>
+      </c>
+      <c r="I42" t="inlineStr">
+        <is>
+          <t>ml</t>
+        </is>
+      </c>
+      <c r="J42" t="inlineStr"/>
+      <c r="K42" t="n">
+        <v>0.125</v>
+      </c>
+      <c r="L42" t="n">
+        <v>0.125</v>
+      </c>
+      <c r="M42" t="inlineStr">
+        <is>
+          <t>(2649, 16)</t>
+        </is>
+      </c>
+      <c r="N42" t="inlineStr">
+        <is>
+          <t>(441, 16)</t>
+        </is>
+      </c>
+      <c r="O42" t="inlineStr">
+        <is>
+          <t>(441, 16)</t>
+        </is>
+      </c>
+      <c r="P42" t="inlineStr">
+        <is>
+          <t>['id_team_away', 'is_cup', 'h2h_35', 'h2h_3_segun_loc', 'h2h_3', 'dif_mean_last_match_goals', 'dif_mean_last_match_goals_against', 'dif_mean_last_match_ball_possession', 'dif_mean_last_match_shots_on_goal', 'dif_mean_last_match_goal_attempts', 'dif_mean_last_match_goal_attempts_against', 'dif_n_player_miss', 'dif_mean_age_player_start', 'dif_mean_hei_player_sub', 'dif_mean_hei_player_miss', 'dif_mean_rat_player_start']</t>
+        </is>
+      </c>
+      <c r="Q42" t="n">
+        <v>10</v>
+      </c>
+      <c r="R42" t="n">
+        <v>56.2358276643991</v>
+      </c>
+      <c r="S42" t="n">
+        <v>50.69913213685511</v>
+      </c>
+      <c r="T42" t="n">
+        <v>47.44292880852345</v>
+      </c>
+      <c r="U42" t="n">
+        <v>56.91609977324264</v>
+      </c>
+      <c r="V42" t="n">
+        <v>-0.6802721088435391</v>
+      </c>
+      <c r="W42" t="n">
+        <v>-0.1120235291660776</v>
+      </c>
+      <c r="X42" t="n">
+        <v>-0.2589641498562218</v>
+      </c>
+      <c r="Y42" t="n">
+        <v>0.02420017005204841</v>
+      </c>
+      <c r="Z42" t="n">
+        <v>0.05995637541050591</v>
+      </c>
+      <c r="AA42" t="n">
+        <v>268.9022489038239</v>
+      </c>
+      <c r="AB42" t="n">
+        <v>0.6097556664485803</v>
+      </c>
+      <c r="AC42" t="n">
+        <v>-0.15</v>
+      </c>
+      <c r="AD42" t="inlineStr">
+        <is>
+          <t>exponential</t>
+        </is>
+      </c>
+      <c r="AE42" t="inlineStr">
+        <is>
+          <t>(0.33, 10)</t>
+        </is>
+      </c>
+      <c r="AF42" t="inlineStr">
+        <is>
+          <t>(1, 50)</t>
+        </is>
+      </c>
+      <c r="AG42" t="inlineStr">
+        <is>
+          <t>SVC</t>
+        </is>
+      </c>
+      <c r="AH42" t="inlineStr">
+        <is>
+          <t>{'C': 0.1, 'break_ties': False, 'cache_size': 200, 'class_weight': None, 'coef0': 0.0, 'decision_function_shape': 'ovo', 'degree': 3, 'gamma': 'scale', 'kernel': 'sigmoid', 'max_iter': -1, 'probability': True, 'random_state': None, 'shrinking': True, 'tol': 0.001, 'verbose': False}</t>
+        </is>
+      </c>
+      <c r="AI42" t="n">
+        <v>56.21212121212121</v>
+      </c>
+      <c r="AJ42" t="n">
+        <v>-0.1549146811799042</v>
+      </c>
+      <c r="AK42" t="n">
+        <v>0.2736442265930763</v>
+      </c>
+      <c r="AL42" t="n">
+        <v>0.9897100994887336</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="n">
+        <v>64</v>
+      </c>
+      <c r="B43" t="n">
+        <v>30</v>
+      </c>
+      <c r="C43" t="n">
+        <v>3</v>
+      </c>
+      <c r="D43" t="b">
+        <v>1</v>
+      </c>
+      <c r="E43" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="F43" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="G43" t="n">
+        <v>10</v>
+      </c>
+      <c r="H43" t="inlineStr">
+        <is>
+          <t>[771, 772, 773]</t>
+        </is>
+      </c>
+      <c r="I43" t="inlineStr">
+        <is>
+          <t>ml</t>
+        </is>
+      </c>
+      <c r="J43" t="inlineStr">
+        <is>
+          <t>under</t>
+        </is>
+      </c>
+      <c r="K43" t="n">
+        <v>0.125</v>
+      </c>
+      <c r="L43" t="n">
+        <v>0.125</v>
+      </c>
+      <c r="M43" t="inlineStr">
+        <is>
+          <t>(1911, 16)</t>
+        </is>
+      </c>
+      <c r="N43" t="inlineStr">
+        <is>
+          <t>(441, 16)</t>
+        </is>
+      </c>
+      <c r="O43" t="inlineStr">
+        <is>
+          <t>(441, 16)</t>
+        </is>
+      </c>
+      <c r="P43" t="inlineStr">
+        <is>
+          <t>['id_team_away', 'is_cup', 'h2h_35', 'h2h_3_segun_loc', 'h2h_3', 'dif_mean_last_match_goals', 'dif_mean_last_match_goals_against', 'dif_mean_last_match_ball_possession', 'dif_mean_last_match_shots_on_goal', 'dif_mean_last_match_goal_attempts', 'dif_mean_last_match_goal_attempts_against', 'dif_n_player_miss', 'dif_mean_age_player_start', 'dif_mean_hei_player_sub', 'dif_mean_hei_player_miss', 'dif_mean_rat_player_start']</t>
+        </is>
+      </c>
+      <c r="Q43" t="n">
+        <v>10</v>
+      </c>
+      <c r="R43" t="n">
+        <v>53.51473922902494</v>
+      </c>
+      <c r="S43" t="n">
+        <v>50.54348145375803</v>
+      </c>
+      <c r="T43" t="n">
+        <v>48.92308259995202</v>
+      </c>
+      <c r="U43" t="n">
+        <v>56.91609977324264</v>
+      </c>
+      <c r="V43" t="n">
+        <v>-3.401360544217695</v>
+      </c>
+      <c r="W43" t="n">
+        <v>-0.1037478371434355</v>
+      </c>
+      <c r="X43" t="n">
+        <v>0.03841642845645112</v>
+      </c>
+      <c r="Y43" t="n">
+        <v>-0.2001612172466357</v>
+      </c>
+      <c r="Z43" t="n">
+        <v>-0.2378778982575852</v>
+      </c>
+      <c r="AA43" t="n">
+        <v>40.34293009019834</v>
+      </c>
+      <c r="AB43" t="n">
+        <v>0.09148056709795541</v>
+      </c>
+      <c r="AC43" t="n">
+        <v>-0.2</v>
+      </c>
+      <c r="AD43" t="inlineStr">
+        <is>
+          <t>exponential</t>
+        </is>
+      </c>
+      <c r="AE43" t="inlineStr">
+        <is>
+          <t>(0.5, 4)</t>
+        </is>
+      </c>
+      <c r="AF43" t="inlineStr">
+        <is>
+          <t>(1, 10)</t>
+        </is>
+      </c>
+      <c r="AG43" t="inlineStr">
+        <is>
+          <t>LogisticRegression</t>
+        </is>
+      </c>
+      <c r="AH43" t="inlineStr">
+        <is>
+          <t>{'C': 0.1, 'class_weight': None, 'dual': False, 'fit_intercept': False, 'intercept_scaling': 1, 'l1_ratio': None, 'max_iter': 1000, 'multi_class': 'auto', 'n_jobs': None, 'penalty': 'l1', 'random_state': None, 'solver': 'liblinear', 'tol': 0.0001, 'verbose': 0, 'warm_start': False}</t>
+        </is>
+      </c>
+      <c r="AI43" t="n">
+        <v>45.70680628272252</v>
+      </c>
+      <c r="AJ43" t="n">
+        <v>-0.2707759196916665</v>
+      </c>
+      <c r="AK43" t="n">
+        <v>-0.1367317823581692</v>
+      </c>
+      <c r="AL43" t="n">
+        <v>-0.01541403277859793</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="n">
+        <v>65</v>
+      </c>
+      <c r="B44" t="n">
+        <v>30</v>
+      </c>
+      <c r="C44" t="n">
+        <v>3</v>
+      </c>
+      <c r="D44" t="b">
+        <v>1</v>
+      </c>
+      <c r="E44" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="F44" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="G44" t="n">
+        <v>10</v>
+      </c>
+      <c r="H44" t="inlineStr">
+        <is>
+          <t>[771, 772, 773]</t>
+        </is>
+      </c>
+      <c r="I44" t="inlineStr"/>
+      <c r="J44" t="inlineStr"/>
+      <c r="K44" t="n">
+        <v>0.125</v>
+      </c>
+      <c r="L44" t="n">
+        <v>0.125</v>
+      </c>
+      <c r="M44" t="inlineStr">
+        <is>
+          <t>(1497, 29)</t>
+        </is>
+      </c>
+      <c r="N44" t="inlineStr">
+        <is>
+          <t>(250, 29)</t>
+        </is>
+      </c>
+      <c r="O44" t="inlineStr">
+        <is>
+          <t>(250, 29)</t>
+        </is>
+      </c>
+      <c r="P44" t="inlineStr">
+        <is>
+          <t>['referee', 'id_team_home', 'id_team_away', 'id_coach_home', 'id_coach_away', 'is_cup', 'h2h_35', 'h2h_3_segun_loc', 'h2h_3', 'dif_mean_last_match_goals', 'dif_mean_last_match_goals_against', 'dif_mean_last_match_fouls', 'dif_mean_last_match_fouls_against', 'dif_mean_last_match_n_matches_last_days_against', 'dif_mean_last_match_ball_possession', 'dif_mean_last_match_points', 'dif_mean_last_match_shots_on_goal', 'dif_mean_last_match_shots_on_goal_against', 'dif_mean_last_match_goal_attempts', 'dif_mean_last_match_goal_attempts_against', 'mean_last_match_mean_rat_player_start_away_against', 'dif_n_player_miss', 'dif_mean_age_player_start', 'dif_mean_age_player_sub', 'dif_mean_hei_player_sub', 'dif_mean_age_player_miss', 'dif_mean_int_rep_player_miss', 'dif_mean_hei_player_miss', 'dif_mean_rat_player_start']</t>
+        </is>
+      </c>
+      <c r="Q44" t="n">
+        <v>10</v>
+      </c>
+      <c r="R44" t="n">
+        <v>57.2</v>
+      </c>
+      <c r="S44" t="n">
+        <v>48.80281959927977</v>
+      </c>
+      <c r="T44" t="n">
+        <v>42.18508535489667</v>
+      </c>
+      <c r="U44" t="n">
+        <v>57.99999999999999</v>
+      </c>
+      <c r="V44" t="n">
+        <v>-0.7999999999999972</v>
+      </c>
+      <c r="W44" t="n">
+        <v>-0.3131592461244961</v>
+      </c>
+      <c r="X44" t="n">
+        <v>-0.1012832790616302</v>
+      </c>
+      <c r="Y44" t="n">
+        <v>0.316393051577138</v>
+      </c>
+      <c r="Z44" t="n">
+        <v>0.2100979903061018</v>
+      </c>
+      <c r="AA44" t="n">
+        <v>51.75373201434827</v>
+      </c>
+      <c r="AB44" t="n">
+        <v>0.2070149280573931</v>
+      </c>
+      <c r="AC44" t="n">
+        <v>-0.05</v>
+      </c>
+      <c r="AD44" t="inlineStr">
+        <is>
+          <t>linear</t>
+        </is>
+      </c>
+      <c r="AE44" t="n">
+        <v>10</v>
+      </c>
+      <c r="AF44" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG44" t="inlineStr">
+        <is>
+          <t>LogisticRegression</t>
+        </is>
+      </c>
+      <c r="AH44" t="inlineStr">
+        <is>
+          <t>{'C': 0.1, 'class_weight': None, 'dual': False, 'fit_intercept': True, 'intercept_scaling': 1, 'l1_ratio': None, 'max_iter': 1000, 'multi_class': 'auto', 'n_jobs': None, 'penalty': 'l1', 'random_state': None, 'solver': 'liblinear', 'tol': 0.0001, 'verbose': 0, 'warm_start': False}</t>
+        </is>
+      </c>
+      <c r="AI44" t="n">
+        <v>55.57046979865773</v>
+      </c>
+      <c r="AJ44" t="n">
+        <v>0.2070149280573931</v>
+      </c>
+      <c r="AK44" t="inlineStr"/>
+      <c r="AL44" t="inlineStr"/>
+    </row>
+    <row r="45">
+      <c r="A45" t="n">
+        <v>66</v>
+      </c>
+      <c r="B45" t="n">
+        <v>30</v>
+      </c>
+      <c r="C45" t="n">
+        <v>3</v>
+      </c>
+      <c r="D45" t="b">
+        <v>1</v>
+      </c>
+      <c r="E45" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="F45" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="G45" t="n">
+        <v>10</v>
+      </c>
+      <c r="H45" t="inlineStr">
+        <is>
+          <t>[771, 772, 773]</t>
+        </is>
+      </c>
+      <c r="I45" t="inlineStr"/>
+      <c r="J45" t="inlineStr">
+        <is>
+          <t>under</t>
+        </is>
+      </c>
+      <c r="K45" t="n">
+        <v>0.125</v>
+      </c>
+      <c r="L45" t="n">
+        <v>0.125</v>
+      </c>
+      <c r="M45" t="inlineStr">
+        <is>
+          <t>(1098, 29)</t>
+        </is>
+      </c>
+      <c r="N45" t="inlineStr">
+        <is>
+          <t>(250, 29)</t>
+        </is>
+      </c>
+      <c r="O45" t="inlineStr">
+        <is>
+          <t>(250, 29)</t>
+        </is>
+      </c>
+      <c r="P45" t="inlineStr">
+        <is>
+          <t>['referee', 'id_team_home', 'id_team_away', 'id_coach_home', 'id_coach_away', 'is_cup', 'h2h_35', 'h2h_3_segun_loc', 'h2h_3', 'dif_mean_last_match_goals', 'dif_mean_last_match_goals_against', 'dif_mean_last_match_fouls', 'dif_mean_last_match_fouls_against', 'dif_mean_last_match_n_matches_last_days_against', 'dif_mean_last_match_ball_possession', 'dif_mean_last_match_points', 'dif_mean_last_match_shots_on_goal', 'dif_mean_last_match_shots_on_goal_against', 'dif_mean_last_match_goal_attempts', 'dif_mean_last_match_goal_attempts_against', 'mean_last_match_mean_rat_player_start_away_against', 'dif_n_player_miss', 'dif_mean_age_player_start', 'dif_mean_age_player_sub', 'dif_mean_hei_player_sub', 'dif_mean_age_player_miss', 'dif_mean_int_rep_player_miss', 'dif_mean_hei_player_miss', 'dif_mean_rat_player_start']</t>
+        </is>
+      </c>
+      <c r="Q45" t="n">
+        <v>10</v>
+      </c>
+      <c r="R45" t="n">
+        <v>56.39999999999999</v>
+      </c>
+      <c r="S45" t="n">
+        <v>55.37545787545787</v>
+      </c>
+      <c r="T45" t="n">
+        <v>55.25524560569648</v>
+      </c>
+      <c r="U45" t="n">
+        <v>54.40000000000001</v>
+      </c>
+      <c r="V45" t="n">
+        <v>1.999999999999986</v>
+      </c>
+      <c r="W45" t="n">
+        <v>0.008365262396943365</v>
+      </c>
+      <c r="X45" t="n">
+        <v>-0.429513932979763</v>
+      </c>
+      <c r="Y45" t="n">
+        <v>1.256100645002409</v>
+      </c>
+      <c r="Z45" t="n">
+        <v>7.2959042112409</v>
+      </c>
+      <c r="AA45" t="n">
+        <v>3352.775895835295</v>
+      </c>
+      <c r="AB45" t="n">
+        <v>13.41110358334118</v>
+      </c>
+      <c r="AC45" t="n">
+        <v>-0.2</v>
+      </c>
+      <c r="AD45" t="inlineStr">
+        <is>
+          <t>linear</t>
+        </is>
+      </c>
+      <c r="AE45" t="n">
+        <v>30</v>
+      </c>
+      <c r="AF45" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG45" t="inlineStr">
+        <is>
+          <t>LogisticRegression</t>
+        </is>
+      </c>
+      <c r="AH45" t="inlineStr">
+        <is>
+          <t>{'C': 0.1, 'class_weight': None, 'dual': False, 'fit_intercept': True, 'intercept_scaling': 1, 'l1_ratio': None, 'max_iter': 1000, 'multi_class': 'auto', 'n_jobs': None, 'penalty': 'l1', 'random_state': None, 'solver': 'saga', 'tol': 0.0001, 'verbose': 0, 'warm_start': False}</t>
+        </is>
+      </c>
+      <c r="AI45" t="n">
+        <v>31.92660550458715</v>
+      </c>
+      <c r="AJ45" t="n">
+        <v>13.41110358334118</v>
+      </c>
+      <c r="AK45" t="inlineStr"/>
+      <c r="AL45" t="inlineStr"/>
+    </row>
+    <row r="46">
+      <c r="A46" t="n">
+        <v>67</v>
+      </c>
+      <c r="B46" t="n">
+        <v>30</v>
+      </c>
+      <c r="C46" t="n">
+        <v>3</v>
+      </c>
+      <c r="D46" t="b">
+        <v>1</v>
+      </c>
+      <c r="E46" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="F46" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="G46" t="n">
+        <v>10</v>
+      </c>
+      <c r="H46" t="inlineStr">
+        <is>
+          <t>[771, 772, 773]</t>
+        </is>
+      </c>
+      <c r="I46" t="inlineStr">
+        <is>
+          <t>ml</t>
+        </is>
+      </c>
+      <c r="J46" t="inlineStr"/>
+      <c r="K46" t="n">
+        <v>0.125</v>
+      </c>
+      <c r="L46" t="n">
+        <v>0.125</v>
+      </c>
+      <c r="M46" t="inlineStr">
+        <is>
+          <t>(2612, 29)</t>
+        </is>
+      </c>
+      <c r="N46" t="inlineStr">
+        <is>
+          <t>(435, 29)</t>
+        </is>
+      </c>
+      <c r="O46" t="inlineStr">
+        <is>
+          <t>(435, 29)</t>
+        </is>
+      </c>
+      <c r="P46" t="inlineStr">
+        <is>
+          <t>['referee', 'id_team_home', 'id_team_away', 'id_coach_home', 'id_coach_away', 'is_cup', 'h2h_35', 'h2h_3_segun_loc', 'h2h_3', 'dif_mean_last_match_goals', 'dif_mean_last_match_goals_against', 'dif_mean_last_match_fouls', 'dif_mean_last_match_fouls_against', 'dif_mean_last_match_n_matches_last_days_against', 'dif_mean_last_match_ball_possession', 'dif_mean_last_match_points', 'dif_mean_last_match_shots_on_goal', 'dif_mean_last_match_shots_on_goal_against', 'dif_mean_last_match_goal_attempts', 'dif_mean_last_match_goal_attempts_against', 'mean_last_match_mean_rat_player_start_away_against', 'dif_n_player_miss', 'dif_mean_age_player_start', 'dif_mean_age_player_sub', 'dif_mean_hei_player_sub', 'dif_mean_age_player_miss', 'dif_mean_int_rep_player_miss', 'dif_mean_hei_player_miss', 'dif_mean_rat_player_start']</t>
+        </is>
+      </c>
+      <c r="Q46" t="n">
+        <v>10</v>
+      </c>
+      <c r="R46" t="n">
+        <v>56.55172413793104</v>
+      </c>
+      <c r="S46" t="n">
+        <v>50.05736337088026</v>
+      </c>
+      <c r="T46" t="n">
+        <v>42.83696673871449</v>
+      </c>
+      <c r="U46" t="n">
+        <v>56.55172413793104</v>
+      </c>
+      <c r="V46" t="n">
+        <v>0</v>
+      </c>
+      <c r="W46" t="n">
+        <v>-0.07899372835915955</v>
+      </c>
+      <c r="X46" t="n">
+        <v>0.1964916353308881</v>
+      </c>
+      <c r="Y46" t="n">
+        <v>0.7094610874620849</v>
+      </c>
+      <c r="Z46" t="n">
+        <v>0.1884243827546652</v>
+      </c>
+      <c r="AA46" t="n">
+        <v>362.582963015212</v>
+      </c>
+      <c r="AB46" t="n">
+        <v>0.8335240529085335</v>
+      </c>
+      <c r="AC46" t="n">
+        <v>-0.05</v>
+      </c>
+      <c r="AD46" t="inlineStr">
+        <is>
+          <t>linear</t>
+        </is>
+      </c>
+      <c r="AE46" t="n">
+        <v>20</v>
+      </c>
+      <c r="AF46" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG46" t="inlineStr">
+        <is>
+          <t>LogisticRegression</t>
+        </is>
+      </c>
+      <c r="AH46" t="inlineStr">
+        <is>
+          <t>{'C': 0.1, 'class_weight': None, 'dual': False, 'fit_intercept': True, 'intercept_scaling': 1, 'l1_ratio': None, 'max_iter': 1000, 'multi_class': 'auto', 'n_jobs': None, 'penalty': 'l1', 'random_state': None, 'solver': 'liblinear', 'tol': 0.0001, 'verbose': 0, 'warm_start': False}</t>
+        </is>
+      </c>
+      <c r="AI46" t="n">
+        <v>55.7088122605364</v>
+      </c>
+      <c r="AJ46" t="n">
+        <v>1.702805546476632</v>
+      </c>
+      <c r="AK46" t="n">
+        <v>0.5633411572836671</v>
+      </c>
+      <c r="AL46" t="n">
+        <v>0.9779296343579632</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="n">
+        <v>68</v>
+      </c>
+      <c r="B47" t="n">
+        <v>30</v>
+      </c>
+      <c r="C47" t="n">
+        <v>3</v>
+      </c>
+      <c r="D47" t="b">
+        <v>1</v>
+      </c>
+      <c r="E47" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="F47" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="G47" t="n">
+        <v>10</v>
+      </c>
+      <c r="H47" t="inlineStr">
+        <is>
+          <t>[771, 772, 773]</t>
+        </is>
+      </c>
+      <c r="I47" t="inlineStr">
+        <is>
+          <t>ml</t>
+        </is>
+      </c>
+      <c r="J47" t="inlineStr">
+        <is>
+          <t>under</t>
+        </is>
+      </c>
+      <c r="K47" t="n">
+        <v>0.125</v>
+      </c>
+      <c r="L47" t="n">
+        <v>0.125</v>
+      </c>
+      <c r="M47" t="inlineStr">
+        <is>
+          <t>(1893, 29)</t>
+        </is>
+      </c>
+      <c r="N47" t="inlineStr">
+        <is>
+          <t>(435, 29)</t>
+        </is>
+      </c>
+      <c r="O47" t="inlineStr">
+        <is>
+          <t>(435, 29)</t>
+        </is>
+      </c>
+      <c r="P47" t="inlineStr">
+        <is>
+          <t>['referee', 'id_team_home', 'id_team_away', 'id_coach_home', 'id_coach_away', 'is_cup', 'h2h_35', 'h2h_3_segun_loc', 'h2h_3', 'dif_mean_last_match_goals', 'dif_mean_last_match_goals_against', 'dif_mean_last_match_fouls', 'dif_mean_last_match_fouls_against', 'dif_mean_last_match_n_matches_last_days_against', 'dif_mean_last_match_ball_possession', 'dif_mean_last_match_points', 'dif_mean_last_match_shots_on_goal', 'dif_mean_last_match_shots_on_goal_against', 'dif_mean_last_match_goal_attempts', 'dif_mean_last_match_goal_attempts_against', 'mean_last_match_mean_rat_player_start_away_against', 'dif_n_player_miss', 'dif_mean_age_player_start', 'dif_mean_age_player_sub', 'dif_mean_hei_player_sub', 'dif_mean_age_player_miss', 'dif_mean_int_rep_player_miss', 'dif_mean_hei_player_miss', 'dif_mean_rat_player_start']</t>
+        </is>
+      </c>
+      <c r="Q47" t="n">
+        <v>10</v>
+      </c>
+      <c r="R47" t="n">
+        <v>51.26436781609195</v>
+      </c>
+      <c r="S47" t="n">
+        <v>49.6333630251027</v>
+      </c>
+      <c r="T47" t="n">
+        <v>49.9829418947066</v>
+      </c>
+      <c r="U47" t="n">
+        <v>56.55172413793104</v>
+      </c>
+      <c r="V47" t="n">
+        <v>-5.287356321839091</v>
+      </c>
+      <c r="W47" t="n">
+        <v>0.9563995441784238</v>
+      </c>
+      <c r="X47" t="n">
+        <v>2.091999803261753</v>
+      </c>
+      <c r="Y47" t="n">
+        <v>2.243262473825937</v>
+      </c>
+      <c r="Z47" t="n">
+        <v>1.705391839010546</v>
+      </c>
+      <c r="AA47" t="n">
+        <v>406.3314767023593</v>
+      </c>
+      <c r="AB47" t="n">
+        <v>0.9340953487410559</v>
+      </c>
+      <c r="AC47" t="n">
+        <v>-0.15</v>
+      </c>
+      <c r="AD47" t="inlineStr">
+        <is>
+          <t>linear</t>
+        </is>
+      </c>
+      <c r="AE47" t="n">
+        <v>20</v>
+      </c>
+      <c r="AF47" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG47" t="inlineStr">
+        <is>
+          <t>LogisticRegression</t>
+        </is>
+      </c>
+      <c r="AH47" t="inlineStr">
+        <is>
+          <t>{'C': 0.1, 'class_weight': None, 'dual': False, 'fit_intercept': True, 'intercept_scaling': 1, 'l1_ratio': None, 'max_iter': 1000, 'multi_class': 'auto', 'n_jobs': None, 'penalty': 'l1', 'random_state': None, 'solver': 'liblinear', 'tol': 0.0001, 'verbose': 0, 'warm_start': False}</t>
+        </is>
+      </c>
+      <c r="AI47" t="n">
+        <v>30.10582010582011</v>
+      </c>
+      <c r="AJ47" t="n">
+        <v>1.260687155366497</v>
+      </c>
+      <c r="AK47" t="n">
+        <v>1.175619375120264</v>
+      </c>
+      <c r="AL47" t="n">
+        <v>1.637837526993139</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="n">
+        <v>69</v>
+      </c>
+      <c r="B48" t="n">
+        <v>30</v>
+      </c>
+      <c r="C48" t="n">
+        <v>3</v>
+      </c>
+      <c r="D48" t="b">
+        <v>1</v>
+      </c>
+      <c r="E48" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="F48" t="inlineStr"/>
+      <c r="G48" t="n">
+        <v>10</v>
+      </c>
+      <c r="H48" t="inlineStr">
+        <is>
+          <t>[771, 772, 773]</t>
+        </is>
+      </c>
+      <c r="I48" t="inlineStr"/>
+      <c r="J48" t="inlineStr"/>
+      <c r="K48" t="n">
+        <v>0.125</v>
+      </c>
+      <c r="L48" t="n">
+        <v>0.125</v>
+      </c>
+      <c r="M48" t="inlineStr">
+        <is>
+          <t>(1495, 34)</t>
+        </is>
+      </c>
+      <c r="N48" t="inlineStr">
+        <is>
+          <t>(250, 34)</t>
+        </is>
+      </c>
+      <c r="O48" t="inlineStr">
+        <is>
+          <t>(250, 34)</t>
+        </is>
+      </c>
+      <c r="P48" t="inlineStr">
+        <is>
+          <t>['referee', 'id_team_home', 'id_team_away', 'id_coach_home', 'id_coach_away', 'is_cup', 'h2h_35', 'h2h_3_segun_loc', 'h2h_3', 'dif_mean_last_match_goals', 'dif_mean_last_match_goals_against', 'dif_mean_last_match_fouls', 'dif_mean_last_match_fouls_against', 'dif_mean_last_match_n_matches_last_days', 'dif_mean_last_match_n_matches_last_days_against', 'dif_mean_last_match_ball_possession', 'dif_mean_last_match_points', 'dif_mean_last_match_shots_on_goal', 'dif_mean_last_match_shots_on_goal_against', 'dif_mean_last_match_goal_attempts', 'dif_mean_last_match_goal_attempts_against', 'mean_last_match_mean_rat_player_start_home_against', 'mean_last_match_mean_rat_player_start_away_against', 'dif_n_player_miss', 'dif_mean_age_player_start', 'dif_mean_age_player_sub', 'dif_mean_hei_player_sub', 'dif_mean_hei_player_start', 'dif_sum_val_player_miss', 'dif_mean_age_player_miss', 'dif_mean_int_rep_player_miss', 'dif_mean_hei_player_miss', 'dif_mean_rat_player_start', 'is_rival_match']</t>
+        </is>
+      </c>
+      <c r="Q48" t="n">
+        <v>10</v>
+      </c>
+      <c r="R48" t="n">
+        <v>56.00000000000001</v>
+      </c>
+      <c r="S48" t="n">
+        <v>48.45230103677184</v>
+      </c>
+      <c r="T48" t="n">
+        <v>42.10615495403906</v>
+      </c>
+      <c r="U48" t="n">
+        <v>57.59999999999999</v>
+      </c>
+      <c r="V48" t="n">
+        <v>-1.599999999999987</v>
+      </c>
+      <c r="W48" t="n">
+        <v>-0.03135652596597851</v>
+      </c>
+      <c r="X48" t="n">
+        <v>-0.08408033502214365</v>
+      </c>
+      <c r="Y48" t="n">
+        <v>-0.06729723141652708</v>
+      </c>
+      <c r="Z48" t="n">
+        <v>-0.03612838687867913</v>
+      </c>
+      <c r="AA48" t="n">
+        <v>-2.712132836197469</v>
+      </c>
+      <c r="AB48" t="n">
+        <v>-0.01084853134478988</v>
+      </c>
+      <c r="AC48" t="n">
+        <v>-0.2</v>
+      </c>
+      <c r="AD48" t="inlineStr">
+        <is>
+          <t>equal</t>
+        </is>
+      </c>
+      <c r="AE48" t="inlineStr">
+        <is>
+          <t>(0, 0)</t>
+        </is>
+      </c>
+      <c r="AF48" t="inlineStr">
+        <is>
+          <t>(1, 0)</t>
+        </is>
+      </c>
+      <c r="AG48" t="inlineStr">
+        <is>
+          <t>LogisticRegression</t>
+        </is>
+      </c>
+      <c r="AH48" t="inlineStr">
+        <is>
+          <t>{'C': 0.1, 'class_weight': None, 'dual': False, 'fit_intercept': True, 'intercept_scaling': 1, 'l1_ratio': None, 'max_iter': 1000, 'multi_class': 'auto', 'n_jobs': None, 'penalty': 'l1', 'random_state': None, 'solver': 'liblinear', 'tol': 0.0001, 'verbose': 0, 'warm_start': False}</t>
+        </is>
+      </c>
+      <c r="AI48" t="n">
+        <v>56.84563758389262</v>
+      </c>
+      <c r="AJ48" t="n">
+        <v>-0.01084853134478988</v>
+      </c>
+      <c r="AK48" t="inlineStr"/>
+      <c r="AL48" t="inlineStr"/>
+    </row>
+    <row r="49">
+      <c r="A49" t="n">
+        <v>70</v>
+      </c>
+      <c r="B49" t="n">
+        <v>30</v>
+      </c>
+      <c r="C49" t="n">
+        <v>3</v>
+      </c>
+      <c r="D49" t="b">
+        <v>1</v>
+      </c>
+      <c r="E49" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="F49" t="inlineStr"/>
+      <c r="G49" t="n">
+        <v>10</v>
+      </c>
+      <c r="H49" t="inlineStr">
+        <is>
+          <t>[771, 772, 773]</t>
+        </is>
+      </c>
+      <c r="I49" t="inlineStr"/>
+      <c r="J49" t="inlineStr">
+        <is>
+          <t>under</t>
+        </is>
+      </c>
+      <c r="K49" t="n">
+        <v>0.125</v>
+      </c>
+      <c r="L49" t="n">
+        <v>0.125</v>
+      </c>
+      <c r="M49" t="inlineStr">
+        <is>
+          <t>(1110, 34)</t>
+        </is>
+      </c>
+      <c r="N49" t="inlineStr">
+        <is>
+          <t>(250, 34)</t>
+        </is>
+      </c>
+      <c r="O49" t="inlineStr">
+        <is>
+          <t>(250, 34)</t>
+        </is>
+      </c>
+      <c r="P49" t="inlineStr">
+        <is>
+          <t>['referee', 'id_team_home', 'id_team_away', 'id_coach_home', 'id_coach_away', 'is_cup', 'h2h_35', 'h2h_3_segun_loc', 'h2h_3', 'dif_mean_last_match_goals', 'dif_mean_last_match_goals_against', 'dif_mean_last_match_fouls', 'dif_mean_last_match_fouls_against', 'dif_mean_last_match_n_matches_last_days', 'dif_mean_last_match_n_matches_last_days_against', 'dif_mean_last_match_ball_possession', 'dif_mean_last_match_points', 'dif_mean_last_match_shots_on_goal', 'dif_mean_last_match_shots_on_goal_against', 'dif_mean_last_match_goal_attempts', 'dif_mean_last_match_goal_attempts_against', 'mean_last_match_mean_rat_player_start_home_against', 'mean_last_match_mean_rat_player_start_away_against', 'dif_n_player_miss', 'dif_mean_age_player_start', 'dif_mean_age_player_sub', 'dif_mean_hei_player_sub', 'dif_mean_hei_player_start', 'dif_sum_val_player_miss', 'dif_mean_age_player_miss', 'dif_mean_int_rep_player_miss', 'dif_mean_hei_player_miss', 'dif_mean_rat_player_start', 'is_rival_match']</t>
+        </is>
+      </c>
+      <c r="Q49" t="n">
+        <v>10</v>
+      </c>
+      <c r="R49" t="n">
+        <v>51.6</v>
+      </c>
+      <c r="S49" t="n">
+        <v>49.63508536993639</v>
+      </c>
+      <c r="T49" t="n">
+        <v>49.97072028108531</v>
+      </c>
+      <c r="U49" t="n">
+        <v>58.8</v>
+      </c>
+      <c r="V49" t="n">
+        <v>-7.199999999999996</v>
+      </c>
+      <c r="W49" t="n">
+        <v>-0.1923166787015577</v>
+      </c>
+      <c r="X49" t="n">
+        <v>-0.3535090663610053</v>
+      </c>
+      <c r="Y49" t="n">
+        <v>0.04271359964487251</v>
+      </c>
+      <c r="Z49" t="n">
+        <v>0.1191083209075636</v>
+      </c>
+      <c r="AA49" t="n">
+        <v>28.22782028276998</v>
+      </c>
+      <c r="AB49" t="n">
+        <v>0.1129112811310799</v>
+      </c>
+      <c r="AC49" t="n">
+        <v>-0.2</v>
+      </c>
+      <c r="AD49" t="inlineStr">
+        <is>
+          <t>linear</t>
+        </is>
+      </c>
+      <c r="AE49" t="n">
+        <v>10</v>
+      </c>
+      <c r="AF49" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG49" t="inlineStr">
+        <is>
+          <t>LogisticRegression</t>
+        </is>
+      </c>
+      <c r="AH49" t="inlineStr">
+        <is>
+          <t>{'C': 0.1, 'class_weight': None, 'dual': False, 'fit_intercept': True, 'intercept_scaling': 1, 'l1_ratio': None, 'max_iter': 1000, 'multi_class': 'auto', 'n_jobs': None, 'penalty': 'l1', 'random_state': None, 'solver': 'liblinear', 'tol': 0.0001, 'verbose': 0, 'warm_start': False}</t>
+        </is>
+      </c>
+      <c r="AI49" t="n">
+        <v>33.33333333333334</v>
+      </c>
+      <c r="AJ49" t="n">
+        <v>0.1129112811310799</v>
+      </c>
+      <c r="AK49" t="inlineStr"/>
+      <c r="AL49" t="inlineStr"/>
+    </row>
+    <row r="50">
+      <c r="A50" t="n">
+        <v>71</v>
+      </c>
+      <c r="B50" t="n">
+        <v>30</v>
+      </c>
+      <c r="C50" t="n">
+        <v>3</v>
+      </c>
+      <c r="D50" t="b">
+        <v>1</v>
+      </c>
+      <c r="E50" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="F50" t="inlineStr"/>
+      <c r="G50" t="n">
+        <v>10</v>
+      </c>
+      <c r="H50" t="inlineStr">
+        <is>
+          <t>[771, 772, 773]</t>
+        </is>
+      </c>
+      <c r="I50" t="inlineStr">
+        <is>
+          <t>ml</t>
+        </is>
+      </c>
+      <c r="J50" t="inlineStr"/>
+      <c r="K50" t="n">
+        <v>0.125</v>
+      </c>
+      <c r="L50" t="n">
+        <v>0.125</v>
+      </c>
+      <c r="M50" t="inlineStr">
+        <is>
+          <t>(2609, 34)</t>
+        </is>
+      </c>
+      <c r="N50" t="inlineStr">
+        <is>
+          <t>(434, 34)</t>
+        </is>
+      </c>
+      <c r="O50" t="inlineStr">
+        <is>
+          <t>(434, 34)</t>
+        </is>
+      </c>
+      <c r="P50" t="inlineStr">
+        <is>
+          <t>['referee', 'id_team_home', 'id_team_away', 'id_coach_home', 'id_coach_away', 'is_cup', 'h2h_35', 'h2h_3_segun_loc', 'h2h_3', 'dif_mean_last_match_goals', 'dif_mean_last_match_goals_against', 'dif_mean_last_match_fouls', 'dif_mean_last_match_fouls_against', 'dif_mean_last_match_n_matches_last_days', 'dif_mean_last_match_n_matches_last_days_against', 'dif_mean_last_match_ball_possession', 'dif_mean_last_match_points', 'dif_mean_last_match_shots_on_goal', 'dif_mean_last_match_shots_on_goal_against', 'dif_mean_last_match_goal_attempts', 'dif_mean_last_match_goal_attempts_against', 'mean_last_match_mean_rat_player_start_home_against', 'mean_last_match_mean_rat_player_start_away_against', 'dif_n_player_miss', 'dif_mean_age_player_start', 'dif_mean_age_player_sub', 'dif_mean_hei_player_sub', 'dif_mean_hei_player_start', 'dif_sum_val_player_miss', 'dif_mean_age_player_miss', 'dif_mean_int_rep_player_miss', 'dif_mean_hei_player_miss', 'dif_mean_rat_player_start', 'is_rival_match']</t>
+        </is>
+      </c>
+      <c r="Q50" t="n">
+        <v>10</v>
+      </c>
+      <c r="R50" t="n">
+        <v>56.68202764976959</v>
+      </c>
+      <c r="S50" t="n">
+        <v>50.54355199282735</v>
+      </c>
+      <c r="T50" t="n">
+        <v>43.17968515377402</v>
+      </c>
+      <c r="U50" t="n">
+        <v>55.99078341013824</v>
+      </c>
+      <c r="V50" t="n">
+        <v>0.6912442396313452</v>
+      </c>
+      <c r="W50" t="n">
+        <v>0.4666472621488916</v>
+      </c>
+      <c r="X50" t="n">
+        <v>0.7028603838677128</v>
+      </c>
+      <c r="Y50" t="n">
+        <v>0.3799890797564625</v>
+      </c>
+      <c r="Z50" t="n">
+        <v>0.8440753367057203</v>
+      </c>
+      <c r="AA50" t="n">
+        <v>148.7898446663614</v>
+      </c>
+      <c r="AB50" t="n">
+        <v>0.3428337434708787</v>
+      </c>
+      <c r="AC50" t="n">
+        <v>-0.05</v>
+      </c>
+      <c r="AD50" t="inlineStr">
+        <is>
+          <t>linear</t>
+        </is>
+      </c>
+      <c r="AE50" t="n">
+        <v>10</v>
+      </c>
+      <c r="AF50" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG50" t="inlineStr">
+        <is>
+          <t>LogisticRegression</t>
+        </is>
+      </c>
+      <c r="AH50" t="inlineStr">
+        <is>
+          <t>{'C': 0.1, 'class_weight': None, 'dual': False, 'fit_intercept': True, 'intercept_scaling': 1, 'l1_ratio': None, 'max_iter': 1000, 'multi_class': 'auto', 'n_jobs': None, 'penalty': 'l1', 'random_state': None, 'solver': 'liblinear', 'tol': 0.0001, 'verbose': 0, 'warm_start': False}</t>
+        </is>
+      </c>
+      <c r="AI50" t="n">
+        <v>54.92307692307692</v>
+      </c>
+      <c r="AJ50" t="n">
+        <v>0.8944246564884503</v>
+      </c>
+      <c r="AK50" t="n">
+        <v>0.5306273554813181</v>
+      </c>
+      <c r="AL50" t="n">
+        <v>0.3538580077311167</v>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="n">
+        <v>72</v>
+      </c>
+      <c r="B51" t="n">
+        <v>30</v>
+      </c>
+      <c r="C51" t="n">
+        <v>3</v>
+      </c>
+      <c r="D51" t="b">
+        <v>1</v>
+      </c>
+      <c r="E51" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="F51" t="inlineStr"/>
+      <c r="G51" t="n">
+        <v>10</v>
+      </c>
+      <c r="H51" t="inlineStr">
+        <is>
+          <t>[771, 772, 773]</t>
+        </is>
+      </c>
+      <c r="I51" t="inlineStr">
+        <is>
+          <t>ml</t>
+        </is>
+      </c>
+      <c r="J51" t="inlineStr">
+        <is>
+          <t>under</t>
+        </is>
+      </c>
+      <c r="K51" t="n">
+        <v>0.125</v>
+      </c>
+      <c r="L51" t="n">
+        <v>0.125</v>
+      </c>
+      <c r="M51" t="inlineStr">
+        <is>
+          <t>(1899, 34)</t>
+        </is>
+      </c>
+      <c r="N51" t="inlineStr">
+        <is>
+          <t>(434, 34)</t>
+        </is>
+      </c>
+      <c r="O51" t="inlineStr">
+        <is>
+          <t>(434, 34)</t>
+        </is>
+      </c>
+      <c r="P51" t="inlineStr">
+        <is>
+          <t>['referee', 'id_team_home', 'id_team_away', 'id_coach_home', 'id_coach_away', 'is_cup', 'h2h_35', 'h2h_3_segun_loc', 'h2h_3', 'dif_mean_last_match_goals', 'dif_mean_last_match_goals_against', 'dif_mean_last_match_fouls', 'dif_mean_last_match_fouls_against', 'dif_mean_last_match_n_matches_last_days', 'dif_mean_last_match_n_matches_last_days_against', 'dif_mean_last_match_ball_possession', 'dif_mean_last_match_points', 'dif_mean_last_match_shots_on_goal', 'dif_mean_last_match_shots_on_goal_against', 'dif_mean_last_match_goal_attempts', 'dif_mean_last_match_goal_attempts_against', 'mean_last_match_mean_rat_player_start_home_against', 'mean_last_match_mean_rat_player_start_away_against', 'dif_n_player_miss', 'dif_mean_age_player_start', 'dif_mean_age_player_sub', 'dif_mean_hei_player_sub', 'dif_mean_hei_player_start', 'dif_sum_val_player_miss', 'dif_mean_age_player_miss', 'dif_mean_int_rep_player_miss', 'dif_mean_hei_player_miss', 'dif_mean_rat_player_start', 'is_rival_match']</t>
+        </is>
+      </c>
+      <c r="Q51" t="n">
+        <v>10</v>
+      </c>
+      <c r="R51" t="n">
+        <v>48.15668202764977</v>
+      </c>
+      <c r="S51" t="n">
+        <v>46.14529324674253</v>
+      </c>
+      <c r="T51" t="n">
+        <v>43.66590595730518</v>
+      </c>
+      <c r="U51" t="n">
+        <v>55.99078341013824</v>
+      </c>
+      <c r="V51" t="n">
+        <v>-7.83410138248847</v>
+      </c>
+      <c r="W51" t="n">
+        <v>-0.3132715603279732</v>
+      </c>
+      <c r="X51" t="n">
+        <v>-0.157847556165686</v>
+      </c>
+      <c r="Y51" t="n">
+        <v>-0.08018831425512189</v>
+      </c>
+      <c r="Z51" t="n">
+        <v>0.135744137241398</v>
+      </c>
+      <c r="AA51" t="n">
+        <v>94.32766131766385</v>
+      </c>
+      <c r="AB51" t="n">
+        <v>0.2173448417457692</v>
+      </c>
+      <c r="AC51" t="n">
+        <v>-0.2</v>
+      </c>
+      <c r="AD51" t="inlineStr">
+        <is>
+          <t>linear</t>
+        </is>
+      </c>
+      <c r="AE51" t="n">
+        <v>10</v>
+      </c>
+      <c r="AF51" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG51" t="inlineStr">
+        <is>
+          <t>SVC</t>
+        </is>
+      </c>
+      <c r="AH51" t="inlineStr">
+        <is>
+          <t>{'C': 0.1, 'break_ties': False, 'cache_size': 200, 'class_weight': None, 'coef0': 0.0, 'decision_function_shape': 'ovo', 'degree': 3, 'gamma': 'scale', 'kernel': 'sigmoid', 'max_iter': -1, 'probability': True, 'random_state': None, 'shrinking': True, 'tol': 0.001, 'verbose': False}</t>
+        </is>
+      </c>
+      <c r="AI51" t="n">
+        <v>15.18518518518518</v>
+      </c>
+      <c r="AJ51" t="n">
+        <v>0.1882272483391918</v>
+      </c>
+      <c r="AK51" t="n">
+        <v>0.1126835893179313</v>
+      </c>
+      <c r="AL51" t="n">
+        <v>0.09098366389263475</v>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="n">
+        <v>73</v>
+      </c>
+      <c r="B52" t="n">
+        <v>30</v>
+      </c>
+      <c r="C52" t="n">
+        <v>3</v>
+      </c>
+      <c r="D52" t="b">
+        <v>1</v>
+      </c>
+      <c r="E52" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="F52" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="G52" t="n">
+        <v>10</v>
+      </c>
+      <c r="H52" t="inlineStr">
+        <is>
+          <t>[771, 772, 773]</t>
+        </is>
+      </c>
+      <c r="I52" t="inlineStr"/>
+      <c r="J52" t="inlineStr"/>
+      <c r="K52" t="n">
+        <v>0.125</v>
+      </c>
+      <c r="L52" t="n">
+        <v>0.125</v>
+      </c>
+      <c r="M52" t="inlineStr">
+        <is>
+          <t>(1740, 19)</t>
+        </is>
+      </c>
+      <c r="N52" t="inlineStr">
+        <is>
+          <t>(290, 19)</t>
+        </is>
+      </c>
+      <c r="O52" t="inlineStr">
+        <is>
+          <t>(290, 19)</t>
+        </is>
+      </c>
+      <c r="P52" t="inlineStr">
+        <is>
+          <t>['id_team_away', 'is_cup', 'h2h_35_segun_loc', 'h2h_35', 'dif_mean_last_match_shots_on_goal', 'dif_mean_last_match_shots_on_goal_against', 'dif_mean_last_match_goal_attempts', 'dif_mean_last_match_goal_attempts_against', 'mean_last_match_mean_rat_player_start_away_against', 'dif_mean_rat_player_sub', 'dif_n_player_miss', 'dif_mean_age_player_start', 'dif_mean_val_player_sub', 'dif_mean_hei_player_sub', 'dif_mean_pot_player_sub', 'dif_mean_hei_player_miss', 'dif_mean_int_rep_player_sub', 'dif_mean_int_rep_player_start', 'dif_mean_rat_player_start']</t>
+        </is>
+      </c>
+      <c r="Q52" t="n">
+        <v>10</v>
+      </c>
+      <c r="R52" t="n">
+        <v>53.79310344827586</v>
+      </c>
+      <c r="S52" t="n">
+        <v>49.34030529453942</v>
+      </c>
+      <c r="T52" t="n">
+        <v>46.68145519077196</v>
+      </c>
+      <c r="U52" t="n">
+        <v>56.55172413793104</v>
+      </c>
+      <c r="V52" t="n">
+        <v>-2.758620689655181</v>
+      </c>
+      <c r="W52" t="n">
+        <v>-0.1818579366604786</v>
+      </c>
+      <c r="X52" t="n">
+        <v>-0.1459458036165533</v>
+      </c>
+      <c r="Y52" t="n">
+        <v>-0.1256587101339899</v>
+      </c>
+      <c r="Z52" t="n">
+        <v>-0.07603093609880154</v>
+      </c>
+      <c r="AA52" t="n">
+        <v>-10.03033158569662</v>
+      </c>
+      <c r="AB52" t="n">
+        <v>-0.03458735029550557</v>
+      </c>
+      <c r="AC52" t="n">
+        <v>-0.5</v>
+      </c>
+      <c r="AD52" t="inlineStr">
+        <is>
+          <t>equal</t>
+        </is>
+      </c>
+      <c r="AE52" t="inlineStr">
+        <is>
+          <t>(0, 0)</t>
+        </is>
+      </c>
+      <c r="AF52" t="inlineStr">
+        <is>
+          <t>(1, 0)</t>
+        </is>
+      </c>
+      <c r="AG52" t="inlineStr">
+        <is>
+          <t>LogisticRegression</t>
+        </is>
+      </c>
+      <c r="AH52" t="inlineStr">
+        <is>
+          <t>{'C': 1, 'class_weight': None, 'dual': False, 'fit_intercept': False, 'intercept_scaling': 1, 'l1_ratio': None, 'max_iter': 1000, 'multi_class': 'auto', 'n_jobs': None, 'penalty': 'l1', 'random_state': None, 'solver': 'saga', 'tol': 0.0001, 'verbose': 0, 'warm_start': False}</t>
+        </is>
+      </c>
+      <c r="AI52" t="n">
+        <v>54.19540229885058</v>
+      </c>
+      <c r="AJ52" t="n">
+        <v>-0.07847890490312597</v>
+      </c>
+      <c r="AK52" t="inlineStr"/>
+      <c r="AL52" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>